<commit_message>
added cors and .gitignore
</commit_message>
<xml_diff>
--- a/StaffingReport.xlsx
+++ b/StaffingReport.xlsx
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2659,19 +2659,19 @@
         <v>129</v>
       </c>
       <c r="I4" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="J4" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="K4" t="n">
-        <v>23.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>433</v>
+        <v>174.1</v>
       </c>
       <c r="M4" t="n">
-        <v>77.09999999999999</v>
+        <v>90.7</v>
       </c>
     </row>
     <row r="5">
@@ -2710,19 +2710,19 @@
         <v>1319</v>
       </c>
       <c r="I5" t="n">
-        <v>1074</v>
+        <v>1239</v>
       </c>
       <c r="J5" t="n">
-        <v>245</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
-        <v>28.9</v>
+        <v>10.7</v>
       </c>
       <c r="L5" t="n">
-        <v>262.3</v>
+        <v>183.8</v>
       </c>
       <c r="M5" t="n">
-        <v>63.9</v>
+        <v>82.2</v>
       </c>
     </row>
     <row r="6">
@@ -2761,19 +2761,19 @@
         <v>82</v>
       </c>
       <c r="I6" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>11</v>
+        <v>3.2</v>
       </c>
       <c r="L6" t="n">
-        <v>403.1</v>
+        <v>98</v>
       </c>
       <c r="M6" t="n">
-        <v>94.90000000000001</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="7">
@@ -2812,19 +2812,19 @@
         <v>119</v>
       </c>
       <c r="I7" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="J7" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>9.9</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>198.9</v>
+        <v>159.1</v>
       </c>
       <c r="M7" t="n">
-        <v>89.3</v>
+        <v>93.59999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -2863,19 +2863,19 @@
         <v>2781</v>
       </c>
       <c r="I8" t="n">
-        <v>2234</v>
+        <v>2663</v>
       </c>
       <c r="J8" t="n">
-        <v>547</v>
+        <v>118</v>
       </c>
       <c r="K8" t="n">
-        <v>33.7</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>183.4</v>
+        <v>145.7</v>
       </c>
       <c r="M8" t="n">
-        <v>52.1</v>
+        <v>86.8</v>
       </c>
     </row>
     <row r="9">
@@ -2914,19 +2914,19 @@
         <v>277</v>
       </c>
       <c r="I9" t="n">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="J9" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="K9" t="n">
-        <v>28.9</v>
+        <v>3.7</v>
       </c>
       <c r="L9" t="n">
-        <v>333.6</v>
+        <v>113.5</v>
       </c>
       <c r="M9" t="n">
-        <v>71.2</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
@@ -2965,19 +2965,19 @@
         <v>142</v>
       </c>
       <c r="I10" t="n">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="J10" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="K10" t="n">
-        <v>27.4</v>
+        <v>14.8</v>
       </c>
       <c r="L10" t="n">
-        <v>250.7</v>
+        <v>182.2</v>
       </c>
       <c r="M10" t="n">
-        <v>73.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -3016,19 +3016,19 @@
         <v>2434</v>
       </c>
       <c r="I11" t="n">
-        <v>2049</v>
+        <v>2325</v>
       </c>
       <c r="J11" t="n">
-        <v>385</v>
+        <v>109</v>
       </c>
       <c r="K11" t="n">
-        <v>24.5</v>
+        <v>5.7</v>
       </c>
       <c r="L11" t="n">
-        <v>165.2</v>
+        <v>114.6</v>
       </c>
       <c r="M11" t="n">
-        <v>60.8</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12">
@@ -3067,19 +3067,19 @@
         <v>241</v>
       </c>
       <c r="I12" t="n">
-        <v>205</v>
+        <v>232</v>
       </c>
       <c r="J12" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="K12" t="n">
-        <v>25.3</v>
+        <v>5.9</v>
       </c>
       <c r="L12" t="n">
-        <v>212.6</v>
+        <v>99</v>
       </c>
       <c r="M12" t="n">
-        <v>75.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -3118,19 +3118,19 @@
         <v>156</v>
       </c>
       <c r="I13" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J13" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="K13" t="n">
-        <v>12.8</v>
+        <v>2.3</v>
       </c>
       <c r="L13" t="n">
-        <v>153.3</v>
+        <v>87.7</v>
       </c>
       <c r="M13" t="n">
-        <v>84.90000000000001</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14">
@@ -3169,19 +3169,19 @@
         <v>2660</v>
       </c>
       <c r="I14" t="n">
-        <v>2106</v>
+        <v>2495</v>
       </c>
       <c r="J14" t="n">
-        <v>554</v>
+        <v>165</v>
       </c>
       <c r="K14" t="n">
-        <v>36.9</v>
+        <v>9.9</v>
       </c>
       <c r="L14" t="n">
-        <v>204.5</v>
+        <v>113.2</v>
       </c>
       <c r="M14" t="n">
-        <v>49.3</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="15">
@@ -3220,19 +3220,19 @@
         <v>257</v>
       </c>
       <c r="I15" t="n">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="J15" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="K15" t="n">
-        <v>22.3</v>
+        <v>6.1</v>
       </c>
       <c r="L15" t="n">
-        <v>227.5</v>
+        <v>134.4</v>
       </c>
       <c r="M15" t="n">
-        <v>73</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -3271,19 +3271,19 @@
         <v>150</v>
       </c>
       <c r="I16" t="n">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="J16" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="K16" t="n">
-        <v>12</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L16" t="n">
-        <v>228.6</v>
+        <v>216.1</v>
       </c>
       <c r="M16" t="n">
-        <v>82</v>
+        <v>89.3</v>
       </c>
     </row>
     <row r="17">
@@ -3322,19 +3322,19 @@
         <v>2476</v>
       </c>
       <c r="I17" t="n">
-        <v>2095</v>
+        <v>2400</v>
       </c>
       <c r="J17" t="n">
-        <v>381</v>
+        <v>76</v>
       </c>
       <c r="K17" t="n">
-        <v>26.3</v>
+        <v>4.5</v>
       </c>
       <c r="L17" t="n">
-        <v>247.8</v>
+        <v>119.8</v>
       </c>
       <c r="M17" t="n">
-        <v>60</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="18">
@@ -3373,19 +3373,19 @@
         <v>232</v>
       </c>
       <c r="I18" t="n">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="J18" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>18</v>
+        <v>5.1</v>
       </c>
       <c r="L18" t="n">
-        <v>187.9</v>
+        <v>146.5</v>
       </c>
       <c r="M18" t="n">
-        <v>80.3</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19">
@@ -3424,19 +3424,19 @@
         <v>153</v>
       </c>
       <c r="I19" t="n">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="J19" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="K19" t="n">
-        <v>23.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L19" t="n">
-        <v>169</v>
+        <v>138.6</v>
       </c>
       <c r="M19" t="n">
-        <v>71.90000000000001</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="20">
@@ -3475,19 +3475,19 @@
         <v>2599</v>
       </c>
       <c r="I20" t="n">
-        <v>2100</v>
+        <v>2479</v>
       </c>
       <c r="J20" t="n">
-        <v>499</v>
+        <v>120</v>
       </c>
       <c r="K20" t="n">
-        <v>34.4</v>
+        <v>7.2</v>
       </c>
       <c r="L20" t="n">
-        <v>179.7</v>
+        <v>145.9</v>
       </c>
       <c r="M20" t="n">
-        <v>48.7</v>
+        <v>86.2</v>
       </c>
     </row>
     <row r="21">
@@ -3526,19 +3526,19 @@
         <v>248</v>
       </c>
       <c r="I21" t="n">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="J21" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="K21" t="n">
-        <v>24.8</v>
+        <v>7.8</v>
       </c>
       <c r="L21" t="n">
-        <v>277.8</v>
+        <v>101.4</v>
       </c>
       <c r="M21" t="n">
-        <v>75.2</v>
+        <v>85.40000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -3577,19 +3577,19 @@
         <v>162</v>
       </c>
       <c r="I22" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="J22" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="K22" t="n">
-        <v>11</v>
+        <v>5.1</v>
       </c>
       <c r="L22" t="n">
-        <v>170.3</v>
+        <v>137.1</v>
       </c>
       <c r="M22" t="n">
-        <v>86.59999999999999</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23">
@@ -3628,19 +3628,19 @@
         <v>2974</v>
       </c>
       <c r="I23" t="n">
-        <v>2412</v>
+        <v>2821</v>
       </c>
       <c r="J23" t="n">
-        <v>562</v>
+        <v>153</v>
       </c>
       <c r="K23" t="n">
-        <v>32.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="L23" t="n">
-        <v>203</v>
+        <v>129.5</v>
       </c>
       <c r="M23" t="n">
-        <v>53.2</v>
+        <v>84.09999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -3679,19 +3679,19 @@
         <v>276</v>
       </c>
       <c r="I24" t="n">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="J24" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="K24" t="n">
-        <v>11.7</v>
+        <v>4.7</v>
       </c>
       <c r="L24" t="n">
-        <v>192.2</v>
+        <v>107.4</v>
       </c>
       <c r="M24" t="n">
-        <v>83.8</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="27">
@@ -3759,16 +3759,16 @@
         <v>1530</v>
       </c>
       <c r="D30" t="n">
-        <v>1257</v>
+        <v>1437</v>
       </c>
       <c r="E30" t="n">
-        <v>273</v>
+        <v>93</v>
       </c>
       <c r="F30" t="n">
-        <v>17.8</v>
+        <v>6.1</v>
       </c>
       <c r="G30" t="n">
-        <v>78.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="H30" t="n">
         <v>51</v>
@@ -3787,16 +3787,16 @@
         <v>3177</v>
       </c>
       <c r="D31" t="n">
-        <v>2573</v>
+        <v>3038</v>
       </c>
       <c r="E31" t="n">
-        <v>604</v>
+        <v>139</v>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
+        <v>4.4</v>
       </c>
       <c r="G31" t="n">
-        <v>70.90000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="H31" t="n">
         <v>88</v>
@@ -3815,16 +3815,16 @@
         <v>2817</v>
       </c>
       <c r="D32" t="n">
-        <v>2364</v>
+        <v>2686</v>
       </c>
       <c r="E32" t="n">
-        <v>451</v>
+        <v>131</v>
       </c>
       <c r="F32" t="n">
-        <v>16</v>
+        <v>4.7</v>
       </c>
       <c r="G32" t="n">
-        <v>69.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="H32" t="n">
         <v>81</v>
@@ -3843,16 +3843,16 @@
         <v>3073</v>
       </c>
       <c r="D33" t="n">
-        <v>2467</v>
+        <v>2888</v>
       </c>
       <c r="E33" t="n">
-        <v>606</v>
+        <v>185</v>
       </c>
       <c r="F33" t="n">
-        <v>19.7</v>
+        <v>6</v>
       </c>
       <c r="G33" t="n">
-        <v>69.09999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="H33" t="n">
         <v>85</v>
@@ -3871,16 +3871,16 @@
         <v>2858</v>
       </c>
       <c r="D34" t="n">
-        <v>2431</v>
+        <v>2769</v>
       </c>
       <c r="E34" t="n">
-        <v>426</v>
+        <v>89</v>
       </c>
       <c r="F34" t="n">
-        <v>14.9</v>
+        <v>3.1</v>
       </c>
       <c r="G34" t="n">
-        <v>74.09999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="H34" t="n">
         <v>83</v>
@@ -3899,16 +3899,16 @@
         <v>3000</v>
       </c>
       <c r="D35" t="n">
-        <v>2442</v>
+        <v>2863</v>
       </c>
       <c r="E35" t="n">
-        <v>557</v>
+        <v>137</v>
       </c>
       <c r="F35" t="n">
-        <v>18.6</v>
+        <v>4.6</v>
       </c>
       <c r="G35" t="n">
-        <v>65.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="H35" t="n">
         <v>86</v>
@@ -3927,16 +3927,16 @@
         <v>3412</v>
       </c>
       <c r="D36" t="n">
-        <v>2795</v>
+        <v>3232</v>
       </c>
       <c r="E36" t="n">
-        <v>614</v>
+        <v>177</v>
       </c>
       <c r="F36" t="n">
-        <v>18</v>
+        <v>5.2</v>
       </c>
       <c r="G36" t="n">
-        <v>74.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="H36" t="n">
         <v>92</v>
@@ -3955,16 +3955,16 @@
         <v>19867</v>
       </c>
       <c r="D37" t="n">
-        <v>16329</v>
+        <v>18913</v>
       </c>
       <c r="E37" t="n">
-        <v>3531</v>
+        <v>951</v>
       </c>
       <c r="F37" t="n">
-        <v>17.8</v>
+        <v>4.8</v>
       </c>
       <c r="G37" t="n">
-        <v>71.8</v>
+        <v>89.3</v>
       </c>
       <c r="H37" t="n">
         <v>566</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G4" t="n">
         <v>129</v>
@@ -4097,19 +4097,19 @@
         <v>129</v>
       </c>
       <c r="I4" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K4" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="L4" t="n">
-        <v>116.1</v>
+        <v>228.3</v>
       </c>
       <c r="M4" t="n">
-        <v>98.40000000000001</v>
+        <v>97.59999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="G5" t="n">
         <v>1319</v>
@@ -4148,19 +4148,19 @@
         <v>1319</v>
       </c>
       <c r="I5" t="n">
-        <v>1299</v>
+        <v>1293</v>
       </c>
       <c r="J5" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="K5" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="L5" t="n">
-        <v>127.1</v>
+        <v>113.8</v>
       </c>
       <c r="M5" t="n">
-        <v>95.8</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="6">
@@ -4190,7 +4190,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
         <v>82</v>
@@ -4199,19 +4199,19 @@
         <v>82</v>
       </c>
       <c r="I6" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
       <c r="L6" t="n">
-        <v>151.2</v>
+        <v>98</v>
       </c>
       <c r="M6" t="n">
-        <v>95.09999999999999</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="7">
@@ -4241,7 +4241,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G7" t="n">
         <v>119</v>
@@ -4256,13 +4256,13 @@
         <v>6</v>
       </c>
       <c r="K7" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L7" t="n">
-        <v>73.7</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>96.5</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="8">
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="G8" t="n">
         <v>2781</v>
@@ -4301,19 +4301,19 @@
         <v>2781</v>
       </c>
       <c r="I8" t="n">
-        <v>2740</v>
+        <v>2749</v>
       </c>
       <c r="J8" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="K8" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L8" t="n">
-        <v>92.7</v>
+        <v>67.5</v>
       </c>
       <c r="M8" t="n">
-        <v>95.8</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="9">
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="G9" t="n">
         <v>277</v>
@@ -4352,19 +4352,19 @@
         <v>277</v>
       </c>
       <c r="I9" t="n">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="L9" t="n">
-        <v>81.5</v>
+        <v>68.3</v>
       </c>
       <c r="M9" t="n">
-        <v>97.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G10" t="n">
         <v>142</v>
@@ -4403,19 +4403,19 @@
         <v>142</v>
       </c>
       <c r="I10" t="n">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3</v>
+        <v>4.5</v>
       </c>
       <c r="L10" t="n">
-        <v>36.3</v>
+        <v>229.9</v>
       </c>
       <c r="M10" t="n">
-        <v>99.3</v>
+        <v>95.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -4445,7 +4445,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G11" t="n">
         <v>2434</v>
@@ -4454,19 +4454,19 @@
         <v>2434</v>
       </c>
       <c r="I11" t="n">
-        <v>2398</v>
+        <v>2379</v>
       </c>
       <c r="J11" t="n">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="K11" t="n">
         <v>2.5</v>
       </c>
       <c r="L11" t="n">
-        <v>71.2</v>
+        <v>88.7</v>
       </c>
       <c r="M11" t="n">
-        <v>95.09999999999999</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="12">
@@ -4496,7 +4496,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G12" t="n">
         <v>241</v>
@@ -4505,19 +4505,19 @@
         <v>241</v>
       </c>
       <c r="I12" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>2.1</v>
+        <v>1.1</v>
       </c>
       <c r="L12" t="n">
-        <v>77.5</v>
+        <v>41.3</v>
       </c>
       <c r="M12" t="n">
-        <v>95.40000000000001</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="13">
@@ -4547,7 +4547,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G13" t="n">
         <v>156</v>
@@ -4556,19 +4556,19 @@
         <v>156</v>
       </c>
       <c r="I13" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K13" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="L13" t="n">
-        <v>115.3</v>
+        <v>87.7</v>
       </c>
       <c r="M13" t="n">
-        <v>96.09999999999999</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14">
@@ -4598,7 +4598,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="G14" t="n">
         <v>2660</v>
@@ -4607,19 +4607,19 @@
         <v>2660</v>
       </c>
       <c r="I14" t="n">
-        <v>2613</v>
+        <v>2622</v>
       </c>
       <c r="J14" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="K14" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="L14" t="n">
-        <v>83.40000000000001</v>
+        <v>56.5</v>
       </c>
       <c r="M14" t="n">
-        <v>96</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="15">
@@ -4649,7 +4649,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G15" t="n">
         <v>257</v>
@@ -4664,10 +4664,10 @@
         <v>5</v>
       </c>
       <c r="K15" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="L15" t="n">
-        <v>98</v>
+        <v>91.7</v>
       </c>
       <c r="M15" t="n">
         <v>96.40000000000001</v>
@@ -4700,7 +4700,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G16" t="n">
         <v>150</v>
@@ -4709,19 +4709,19 @@
         <v>150</v>
       </c>
       <c r="I16" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="L16" t="n">
-        <v>95.09999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>97.3</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="17">
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="G17" t="n">
         <v>2476</v>
@@ -4760,19 +4760,19 @@
         <v>2476</v>
       </c>
       <c r="I17" t="n">
-        <v>2439</v>
+        <v>2437</v>
       </c>
       <c r="J17" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K17" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="L17" t="n">
-        <v>78.3</v>
+        <v>113.2</v>
       </c>
       <c r="M17" t="n">
-        <v>95.09999999999999</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="18">
@@ -4802,7 +4802,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G18" t="n">
         <v>232</v>
@@ -4817,13 +4817,13 @@
         <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="L18" t="n">
-        <v>106.4</v>
+        <v>122</v>
       </c>
       <c r="M18" t="n">
-        <v>97.8</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -4853,7 +4853,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G19" t="n">
         <v>153</v>
@@ -4862,19 +4862,19 @@
         <v>153</v>
       </c>
       <c r="I19" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="J19" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>1.7</v>
       </c>
       <c r="L19" t="n">
-        <v>154.9</v>
+        <v>120.8</v>
       </c>
       <c r="M19" t="n">
-        <v>95.8</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
@@ -4904,7 +4904,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="G20" t="n">
         <v>2599</v>
@@ -4913,19 +4913,19 @@
         <v>2599</v>
       </c>
       <c r="I20" t="n">
-        <v>2564</v>
+        <v>2556</v>
       </c>
       <c r="J20" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="K20" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="L20" t="n">
-        <v>80</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>95.3</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="21">
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="G21" t="n">
         <v>248</v>
@@ -4970,13 +4970,13 @@
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="L21" t="n">
-        <v>56.3</v>
+        <v>46.4</v>
       </c>
       <c r="M21" t="n">
-        <v>99.59999999999999</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="22">
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G22" t="n">
         <v>162</v>
@@ -5015,19 +5015,19 @@
         <v>162</v>
       </c>
       <c r="I22" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>0.2</v>
       </c>
       <c r="L22" t="n">
-        <v>160.3</v>
+        <v>17.1</v>
       </c>
       <c r="M22" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="G23" t="n">
         <v>2974</v>
@@ -5066,19 +5066,19 @@
         <v>2974</v>
       </c>
       <c r="I23" t="n">
-        <v>2942</v>
+        <v>2946</v>
       </c>
       <c r="J23" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="K23" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="L23" t="n">
-        <v>67.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>96.2</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -5108,7 +5108,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G24" t="n">
         <v>276</v>
@@ -5117,19 +5117,19 @@
         <v>276</v>
       </c>
       <c r="I24" t="n">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K24" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="L24" t="n">
-        <v>93.7</v>
+        <v>105.2</v>
       </c>
       <c r="M24" t="n">
-        <v>95.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -5197,19 +5197,19 @@
         <v>1530</v>
       </c>
       <c r="D30" t="n">
-        <v>1506</v>
+        <v>1496</v>
       </c>
       <c r="E30" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="G30" t="n">
         <v>96.40000000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31">
@@ -5225,19 +5225,19 @@
         <v>3177</v>
       </c>
       <c r="D31" t="n">
-        <v>3126</v>
+        <v>3133</v>
       </c>
       <c r="E31" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F31" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="G31" t="n">
-        <v>96.5</v>
+        <v>96</v>
       </c>
       <c r="H31" t="n">
-        <v>135</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32">
@@ -5253,19 +5253,19 @@
         <v>2817</v>
       </c>
       <c r="D32" t="n">
-        <v>2778</v>
+        <v>2755</v>
       </c>
       <c r="E32" t="n">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F32" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>96.59999999999999</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H32" t="n">
-        <v>120</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33">
@@ -5281,19 +5281,19 @@
         <v>3073</v>
       </c>
       <c r="D33" t="n">
-        <v>3017</v>
+        <v>3024</v>
       </c>
       <c r="E33" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="F33" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="G33" t="n">
         <v>96.2</v>
       </c>
       <c r="H33" t="n">
-        <v>133</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34">
@@ -5309,19 +5309,19 @@
         <v>2858</v>
       </c>
       <c r="D34" t="n">
-        <v>2814</v>
+        <v>2811</v>
       </c>
       <c r="E34" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F34" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="G34" t="n">
-        <v>96.7</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H34" t="n">
-        <v>124</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35">
@@ -5337,19 +5337,19 @@
         <v>3000</v>
       </c>
       <c r="D35" t="n">
-        <v>2955</v>
+        <v>2950</v>
       </c>
       <c r="E35" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F35" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G35" t="n">
-        <v>96.90000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="H35" t="n">
-        <v>131</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36">
@@ -5365,19 +5365,19 @@
         <v>3412</v>
       </c>
       <c r="D36" t="n">
-        <v>3371</v>
+        <v>3373</v>
       </c>
       <c r="E36" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F36" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G36" t="n">
-        <v>95.7</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>144</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37">
@@ -5393,19 +5393,19 @@
         <v>19867</v>
       </c>
       <c r="D37" t="n">
-        <v>19567</v>
+        <v>19542</v>
       </c>
       <c r="E37" t="n">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="F37" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="G37" t="n">
-        <v>96.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="H37" t="n">
-        <v>869</v>
+        <v>636</v>
       </c>
     </row>
     <row r="40">
@@ -5465,19 +5465,19 @@
         <v>51</v>
       </c>
       <c r="C43" t="n">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="D43" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>78.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="F43" t="n">
         <v>96.40000000000001</v>
       </c>
       <c r="G43" t="n">
-        <v>17.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="44">
@@ -5490,19 +5490,19 @@
         <v>88</v>
       </c>
       <c r="C44" t="n">
-        <v>135</v>
+        <v>98</v>
       </c>
       <c r="D44" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E44" t="n">
-        <v>70.90000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="F44" t="n">
-        <v>96.5</v>
+        <v>96</v>
       </c>
       <c r="G44" t="n">
-        <v>25.6</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="45">
@@ -5515,19 +5515,19 @@
         <v>81</v>
       </c>
       <c r="C45" t="n">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="D45" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>69.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="F45" t="n">
-        <v>96.59999999999999</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G45" t="n">
-        <v>26.8</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -5540,19 +5540,19 @@
         <v>85</v>
       </c>
       <c r="C46" t="n">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="D46" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="E46" t="n">
-        <v>69.09999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="F46" t="n">
         <v>96.2</v>
       </c>
       <c r="G46" t="n">
-        <v>27.1</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="47">
@@ -5565,19 +5565,19 @@
         <v>83</v>
       </c>
       <c r="C47" t="n">
-        <v>124</v>
+        <v>91</v>
       </c>
       <c r="D47" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E47" t="n">
-        <v>74.09999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="F47" t="n">
-        <v>96.7</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>22.6</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="48">
@@ -5590,19 +5590,19 @@
         <v>86</v>
       </c>
       <c r="C48" t="n">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="D48" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E48" t="n">
-        <v>65.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="F48" t="n">
-        <v>96.90000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="G48" t="n">
-        <v>31.6</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="49">
@@ -5615,19 +5615,19 @@
         <v>92</v>
       </c>
       <c r="C49" t="n">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="D49" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="E49" t="n">
-        <v>74.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="F49" t="n">
-        <v>95.7</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G49" t="n">
-        <v>21.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="50">
@@ -5640,19 +5640,19 @@
         <v>566</v>
       </c>
       <c r="C50" t="n">
-        <v>869</v>
+        <v>636</v>
       </c>
       <c r="D50" t="n">
-        <v>303</v>
+        <v>70</v>
       </c>
       <c r="E50" t="n">
-        <v>71.8</v>
+        <v>89.3</v>
       </c>
       <c r="F50" t="n">
-        <v>96.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="G50" t="n">
-        <v>24.7</v>
+        <v>7.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the simulation for different sla range and utilization to campare the agent needs for different sla's
</commit_message>
<xml_diff>
--- a/StaffingReport.xlsx
+++ b/StaffingReport.xlsx
@@ -496,28 +496,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>184</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>210</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>218</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>224</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>241</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>237</v>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="5">
@@ -527,28 +527,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>151</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>151</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>191</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>179</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>182</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>170</v>
       </c>
       <c r="I5" t="n">
-        <v>19</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="6">
@@ -558,28 +558,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>185</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>148</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>141</v>
       </c>
       <c r="I6" t="n">
-        <v>14</v>
+        <v>917</v>
       </c>
     </row>
     <row r="7">
@@ -589,28 +589,28 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>106</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>129</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>116</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>122</v>
       </c>
       <c r="I7" t="n">
-        <v>14</v>
+        <v>720</v>
       </c>
     </row>
     <row r="8">
@@ -620,28 +620,28 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>106</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>88</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="I8" t="n">
-        <v>10</v>
+        <v>570</v>
       </c>
     </row>
     <row r="9">
@@ -651,28 +651,28 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>91</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>87</v>
       </c>
       <c r="I9" t="n">
-        <v>15</v>
+        <v>525</v>
       </c>
     </row>
     <row r="10">
@@ -682,28 +682,28 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>92</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>149</v>
       </c>
       <c r="I10" t="n">
-        <v>16</v>
+        <v>648</v>
       </c>
     </row>
     <row r="11">
@@ -713,28 +713,28 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>111</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>91</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>110</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>120</v>
       </c>
       <c r="H11" t="n">
-        <v>6</v>
+        <v>116</v>
       </c>
       <c r="I11" t="n">
-        <v>30</v>
+        <v>679</v>
       </c>
     </row>
     <row r="12">
@@ -744,28 +744,28 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>108</v>
       </c>
       <c r="C12" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>98</v>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="F12" t="n">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="G12" t="n">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="H12" t="n">
-        <v>16</v>
+        <v>115</v>
       </c>
       <c r="I12" t="n">
-        <v>76</v>
+        <v>683</v>
       </c>
     </row>
     <row r="13">
@@ -775,28 +775,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="C13" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D13" t="n">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="E13" t="n">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="F13" t="n">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="G13" t="n">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="H13" t="n">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="I13" t="n">
-        <v>233</v>
+        <v>590</v>
       </c>
     </row>
     <row r="14">
@@ -806,28 +806,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C14" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E14" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F14" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G14" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H14" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I14" t="n">
-        <v>617</v>
+        <v>596</v>
       </c>
     </row>
     <row r="15">
@@ -837,28 +837,28 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>142</v>
+        <v>105</v>
       </c>
       <c r="C15" t="n">
-        <v>176</v>
+        <v>27</v>
       </c>
       <c r="D15" t="n">
-        <v>172</v>
+        <v>112</v>
       </c>
       <c r="E15" t="n">
-        <v>189</v>
+        <v>111</v>
       </c>
       <c r="F15" t="n">
-        <v>183</v>
+        <v>121</v>
       </c>
       <c r="G15" t="n">
-        <v>203</v>
+        <v>124</v>
       </c>
       <c r="H15" t="n">
-        <v>212</v>
+        <v>121</v>
       </c>
       <c r="I15" t="n">
-        <v>1277</v>
+        <v>721</v>
       </c>
     </row>
     <row r="16">
@@ -868,28 +868,28 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>225</v>
+        <v>103</v>
       </c>
       <c r="C16" t="n">
-        <v>320</v>
+        <v>36</v>
       </c>
       <c r="D16" t="n">
-        <v>314</v>
+        <v>127</v>
       </c>
       <c r="E16" t="n">
-        <v>340</v>
+        <v>130</v>
       </c>
       <c r="F16" t="n">
-        <v>329</v>
+        <v>132</v>
       </c>
       <c r="G16" t="n">
-        <v>316</v>
+        <v>167</v>
       </c>
       <c r="H16" t="n">
-        <v>380</v>
+        <v>142</v>
       </c>
       <c r="I16" t="n">
-        <v>2224</v>
+        <v>837</v>
       </c>
     </row>
     <row r="17">
@@ -899,28 +899,28 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>258</v>
+        <v>104</v>
       </c>
       <c r="C17" t="n">
-        <v>482</v>
+        <v>50</v>
       </c>
       <c r="D17" t="n">
-        <v>442</v>
+        <v>132</v>
       </c>
       <c r="E17" t="n">
-        <v>451</v>
+        <v>151</v>
       </c>
       <c r="F17" t="n">
-        <v>446</v>
+        <v>159</v>
       </c>
       <c r="G17" t="n">
-        <v>436</v>
+        <v>160</v>
       </c>
       <c r="H17" t="n">
-        <v>519</v>
+        <v>151</v>
       </c>
       <c r="I17" t="n">
-        <v>3034</v>
+        <v>907</v>
       </c>
     </row>
     <row r="18">
@@ -930,28 +930,28 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>228</v>
+        <v>99</v>
       </c>
       <c r="C18" t="n">
-        <v>473</v>
+        <v>68</v>
       </c>
       <c r="D18" t="n">
-        <v>416</v>
+        <v>151</v>
       </c>
       <c r="E18" t="n">
-        <v>437</v>
+        <v>163</v>
       </c>
       <c r="F18" t="n">
-        <v>429</v>
+        <v>175</v>
       </c>
       <c r="G18" t="n">
-        <v>452</v>
+        <v>176</v>
       </c>
       <c r="H18" t="n">
-        <v>502</v>
+        <v>159</v>
       </c>
       <c r="I18" t="n">
-        <v>2937</v>
+        <v>991</v>
       </c>
     </row>
     <row r="19">
@@ -961,28 +961,28 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>169</v>
+        <v>99</v>
       </c>
       <c r="C19" t="n">
-        <v>422</v>
+        <v>107</v>
       </c>
       <c r="D19" t="n">
-        <v>367</v>
+        <v>193</v>
       </c>
       <c r="E19" t="n">
-        <v>405</v>
+        <v>185</v>
       </c>
       <c r="F19" t="n">
-        <v>358</v>
+        <v>197</v>
       </c>
       <c r="G19" t="n">
-        <v>395</v>
+        <v>336</v>
       </c>
       <c r="H19" t="n">
-        <v>470</v>
+        <v>204</v>
       </c>
       <c r="I19" t="n">
-        <v>2586</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="20">
@@ -992,28 +992,28 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>134</v>
+        <v>95</v>
       </c>
       <c r="C20" t="n">
-        <v>380</v>
+        <v>178</v>
       </c>
       <c r="D20" t="n">
-        <v>317</v>
+        <v>223</v>
       </c>
       <c r="E20" t="n">
-        <v>362</v>
+        <v>251</v>
       </c>
       <c r="F20" t="n">
-        <v>315</v>
+        <v>269</v>
       </c>
       <c r="G20" t="n">
-        <v>351</v>
+        <v>277</v>
       </c>
       <c r="H20" t="n">
-        <v>372</v>
+        <v>238</v>
       </c>
       <c r="I20" t="n">
-        <v>2231</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="21">
@@ -1023,28 +1023,28 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C21" t="n">
+        <v>233</v>
+      </c>
+      <c r="D21" t="n">
+        <v>266</v>
+      </c>
+      <c r="E21" t="n">
+        <v>307</v>
+      </c>
+      <c r="F21" t="n">
+        <v>296</v>
+      </c>
+      <c r="G21" t="n">
         <v>303</v>
       </c>
-      <c r="D21" t="n">
-        <v>245</v>
-      </c>
-      <c r="E21" t="n">
-        <v>277</v>
-      </c>
-      <c r="F21" t="n">
-        <v>243</v>
-      </c>
-      <c r="G21" t="n">
-        <v>267</v>
-      </c>
       <c r="H21" t="n">
-        <v>312</v>
+        <v>261</v>
       </c>
       <c r="I21" t="n">
-        <v>1745</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="22">
@@ -1054,28 +1054,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="C22" t="n">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="D22" t="n">
-        <v>161</v>
+        <v>261</v>
       </c>
       <c r="E22" t="n">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="F22" t="n">
-        <v>173</v>
+        <v>282</v>
       </c>
       <c r="G22" t="n">
-        <v>179</v>
+        <v>326</v>
       </c>
       <c r="H22" t="n">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="I22" t="n">
-        <v>1209</v>
+        <v>1697</v>
       </c>
     </row>
     <row r="23">
@@ -1085,28 +1085,28 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C23" t="n">
-        <v>129</v>
+        <v>250</v>
       </c>
       <c r="D23" t="n">
-        <v>117</v>
+        <v>285</v>
       </c>
       <c r="E23" t="n">
-        <v>128</v>
+        <v>309</v>
       </c>
       <c r="F23" t="n">
-        <v>110</v>
+        <v>304</v>
       </c>
       <c r="G23" t="n">
-        <v>122</v>
+        <v>293</v>
       </c>
       <c r="H23" t="n">
-        <v>123</v>
+        <v>252</v>
       </c>
       <c r="I23" t="n">
-        <v>759</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="24">
@@ -1116,28 +1116,28 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="C24" t="n">
-        <v>75</v>
+        <v>323</v>
       </c>
       <c r="D24" t="n">
-        <v>66</v>
+        <v>345</v>
       </c>
       <c r="E24" t="n">
-        <v>66</v>
+        <v>367</v>
       </c>
       <c r="F24" t="n">
-        <v>61</v>
+        <v>368</v>
       </c>
       <c r="G24" t="n">
-        <v>66</v>
+        <v>355</v>
       </c>
       <c r="H24" t="n">
-        <v>78</v>
+        <v>302</v>
       </c>
       <c r="I24" t="n">
-        <v>433</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="25">
@@ -1147,28 +1147,28 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="C25" t="n">
-        <v>36</v>
+        <v>311</v>
       </c>
       <c r="D25" t="n">
-        <v>24</v>
+        <v>331</v>
       </c>
       <c r="E25" t="n">
-        <v>32</v>
+        <v>333</v>
       </c>
       <c r="F25" t="n">
-        <v>28</v>
+        <v>356</v>
       </c>
       <c r="G25" t="n">
-        <v>32</v>
+        <v>341</v>
       </c>
       <c r="H25" t="n">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="I25" t="n">
-        <v>198</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="26">
@@ -1178,28 +1178,28 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="C26" t="n">
-        <v>21</v>
+        <v>279</v>
       </c>
       <c r="D26" t="n">
-        <v>17</v>
+        <v>333</v>
       </c>
       <c r="E26" t="n">
-        <v>16</v>
+        <v>342</v>
       </c>
       <c r="F26" t="n">
-        <v>14</v>
+        <v>323</v>
       </c>
       <c r="G26" t="n">
-        <v>15</v>
+        <v>301</v>
       </c>
       <c r="H26" t="n">
-        <v>20</v>
+        <v>256</v>
       </c>
       <c r="I26" t="n">
-        <v>108</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="27">
@@ -1209,28 +1209,28 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>264</v>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>312</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>315</v>
       </c>
       <c r="F27" t="n">
-        <v>6</v>
+        <v>312</v>
       </c>
       <c r="G27" t="n">
-        <v>8</v>
+        <v>296</v>
       </c>
       <c r="H27" t="n">
-        <v>9</v>
+        <v>239</v>
       </c>
       <c r="I27" t="n">
-        <v>52</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="28">
@@ -1240,28 +1240,28 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1530</v>
+        <v>2399</v>
       </c>
       <c r="C28" t="n">
-        <v>3177</v>
+        <v>2604</v>
       </c>
       <c r="D28" t="n">
-        <v>2817</v>
+        <v>4259</v>
       </c>
       <c r="E28" t="n">
-        <v>3073</v>
+        <v>4659</v>
       </c>
       <c r="F28" t="n">
-        <v>2858</v>
+        <v>4633</v>
       </c>
       <c r="G28" t="n">
-        <v>3000</v>
+        <v>4903</v>
       </c>
       <c r="H28" t="n">
-        <v>3412</v>
+        <v>4295</v>
       </c>
       <c r="I28" t="n">
-        <v>19867</v>
+        <v>27752</v>
       </c>
     </row>
     <row r="31">
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41">
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43">
@@ -1449,25 +1449,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -1477,25 +1477,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -1505,25 +1505,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -1533,25 +1533,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -1561,25 +1561,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -1589,25 +1589,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -1617,25 +1617,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1645,25 +1645,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -1673,25 +1673,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -1701,25 +1701,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H11" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -1729,25 +1729,25 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" t="n">
         <v>12</v>
       </c>
-      <c r="C12" t="n">
-        <v>12</v>
-      </c>
-      <c r="D12" t="n">
-        <v>12</v>
-      </c>
-      <c r="E12" t="n">
-        <v>13</v>
-      </c>
-      <c r="F12" t="n">
-        <v>13</v>
-      </c>
-      <c r="G12" t="n">
-        <v>15</v>
-      </c>
       <c r="H12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -1757,25 +1757,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G13" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="H13" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -1785,25 +1785,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G14" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="H14" t="n">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -1813,25 +1813,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="E15" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="F15" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="G15" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="H15" t="n">
-        <v>62</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -1841,25 +1841,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="E16" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="G16" t="n">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="H16" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -1869,25 +1869,25 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="E17" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="F17" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="G17" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="H17" t="n">
-        <v>56</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18">
@@ -1897,25 +1897,25 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="D18" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="E18" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="F18" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="G18" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="H18" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -1925,25 +1925,25 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D19" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E19" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F19" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G19" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H19" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20">
@@ -1956,19 +1956,19 @@
         <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D20" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E20" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F20" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G20" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H20" t="n">
         <v>27</v>
@@ -1981,25 +1981,25 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F21" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="G21" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="H21" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22">
@@ -2009,25 +2009,25 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F22" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G22" t="n">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="H22" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23">
@@ -2037,25 +2037,25 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24">
@@ -2065,25 +2065,25 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="G24" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25">
@@ -2093,25 +2093,25 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="H25" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2165,13 +2165,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>566</v>
+        <v>526</v>
       </c>
       <c r="C4" t="n">
-        <v>4528</v>
+        <v>4208</v>
       </c>
       <c r="D4" t="n">
-        <v>58.5</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
@@ -2301,31 +2301,31 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C16" t="n">
-        <v>408</v>
+        <v>360</v>
       </c>
       <c r="D16" t="n">
-        <v>56.1</v>
+        <v>76.7</v>
       </c>
       <c r="E16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F16" t="n">
+        <v>104</v>
+      </c>
+      <c r="G16" t="n">
         <v>12</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H16" t="n">
         <v>96</v>
       </c>
-      <c r="G16" t="n">
-        <v>33</v>
-      </c>
-      <c r="H16" t="n">
-        <v>264</v>
-      </c>
       <c r="I16" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="J16" t="n">
-        <v>48</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17">
@@ -2335,31 +2335,31 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="C17" t="n">
-        <v>704</v>
+        <v>512</v>
       </c>
       <c r="D17" t="n">
-        <v>59.7</v>
+        <v>57.8</v>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>96</v>
+        <v>32</v>
       </c>
       <c r="G17" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="H17" t="n">
-        <v>464</v>
+        <v>200</v>
       </c>
       <c r="I17" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="J17" t="n">
-        <v>144</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18">
@@ -2369,13 +2369,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C18" t="n">
-        <v>648</v>
+        <v>624</v>
       </c>
       <c r="D18" t="n">
-        <v>58.3</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="E18" t="n">
         <v>12</v>
@@ -2384,16 +2384,16 @@
         <v>96</v>
       </c>
       <c r="G18" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="H18" t="n">
-        <v>424</v>
+        <v>232</v>
       </c>
       <c r="I18" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J18" t="n">
-        <v>128</v>
+        <v>296</v>
       </c>
     </row>
     <row r="19">
@@ -2403,31 +2403,31 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C19" t="n">
-        <v>680</v>
+        <v>704</v>
       </c>
       <c r="D19" t="n">
-        <v>59.6</v>
+        <v>73</v>
       </c>
       <c r="E19" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="G19" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="H19" t="n">
-        <v>432</v>
+        <v>264</v>
       </c>
       <c r="I19" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J19" t="n">
-        <v>144</v>
+        <v>320</v>
       </c>
     </row>
     <row r="20">
@@ -2437,13 +2437,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C20" t="n">
-        <v>664</v>
+        <v>680</v>
       </c>
       <c r="D20" t="n">
-        <v>57.7</v>
+        <v>75.3</v>
       </c>
       <c r="E20" t="n">
         <v>13</v>
@@ -2452,16 +2452,16 @@
         <v>104</v>
       </c>
       <c r="G20" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="H20" t="n">
-        <v>432</v>
+        <v>256</v>
       </c>
       <c r="I20" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="J20" t="n">
-        <v>128</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21">
@@ -2471,31 +2471,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C21" t="n">
-        <v>688</v>
+        <v>704</v>
       </c>
       <c r="D21" t="n">
-        <v>57.7</v>
+        <v>76.7</v>
       </c>
       <c r="E21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F21" t="n">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="G21" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="H21" t="n">
-        <v>432</v>
+        <v>288</v>
       </c>
       <c r="I21" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J21" t="n">
-        <v>136</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22">
@@ -2505,31 +2505,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C22" t="n">
-        <v>736</v>
+        <v>624</v>
       </c>
       <c r="D22" t="n">
-        <v>60.2</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F22" t="n">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="G22" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="H22" t="n">
-        <v>496</v>
+        <v>224</v>
       </c>
       <c r="I22" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="J22" t="n">
-        <v>136</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -2650,28 +2650,28 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G4" t="n">
-        <v>129</v>
+        <v>782</v>
       </c>
       <c r="H4" t="n">
-        <v>129</v>
+        <v>782</v>
       </c>
       <c r="I4" t="n">
-        <v>118</v>
+        <v>637</v>
       </c>
       <c r="J4" t="n">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="K4" t="n">
-        <v>8.300000000000001</v>
+        <v>28.3</v>
       </c>
       <c r="L4" t="n">
-        <v>174.1</v>
+        <v>264.9</v>
       </c>
       <c r="M4" t="n">
-        <v>90.7</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="5">
@@ -2701,28 +2701,28 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>1319</v>
+        <v>795</v>
       </c>
       <c r="H5" t="n">
-        <v>1319</v>
+        <v>795</v>
       </c>
       <c r="I5" t="n">
-        <v>1239</v>
+        <v>578</v>
       </c>
       <c r="J5" t="n">
-        <v>80</v>
+        <v>217</v>
       </c>
       <c r="K5" t="n">
-        <v>10.7</v>
+        <v>53.7</v>
       </c>
       <c r="L5" t="n">
-        <v>183.8</v>
+        <v>370.4</v>
       </c>
       <c r="M5" t="n">
-        <v>82.2</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="6">
@@ -2752,28 +2752,28 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="H6" t="n">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>759</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="K6" t="n">
-        <v>3.2</v>
+        <v>11.5</v>
       </c>
       <c r="L6" t="n">
-        <v>98</v>
+        <v>210.2</v>
       </c>
       <c r="M6" t="n">
-        <v>96.2</v>
+        <v>83.7</v>
       </c>
     </row>
     <row r="7">
@@ -2803,28 +2803,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G7" t="n">
-        <v>119</v>
+        <v>167</v>
       </c>
       <c r="H7" t="n">
-        <v>119</v>
+        <v>167</v>
       </c>
       <c r="I7" t="n">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="J7" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>14.1</v>
       </c>
       <c r="L7" t="n">
-        <v>159.1</v>
+        <v>284.4</v>
       </c>
       <c r="M7" t="n">
-        <v>93.59999999999999</v>
+        <v>89.3</v>
       </c>
     </row>
     <row r="8">
@@ -2854,28 +2854,28 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
-        <v>2781</v>
+        <v>913</v>
       </c>
       <c r="H8" t="n">
-        <v>2781</v>
+        <v>913</v>
       </c>
       <c r="I8" t="n">
-        <v>2663</v>
+        <v>788</v>
       </c>
       <c r="J8" t="n">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="K8" t="n">
-        <v>7</v>
+        <v>18.9</v>
       </c>
       <c r="L8" t="n">
-        <v>145.7</v>
+        <v>207</v>
       </c>
       <c r="M8" t="n">
-        <v>86.8</v>
+        <v>72.09999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -2905,28 +2905,28 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="G9" t="n">
-        <v>277</v>
+        <v>1524</v>
       </c>
       <c r="H9" t="n">
-        <v>277</v>
+        <v>1524</v>
       </c>
       <c r="I9" t="n">
-        <v>266</v>
+        <v>1244</v>
       </c>
       <c r="J9" t="n">
-        <v>11</v>
+        <v>280</v>
       </c>
       <c r="K9" t="n">
-        <v>3.7</v>
+        <v>34.6</v>
       </c>
       <c r="L9" t="n">
-        <v>113.5</v>
+        <v>180.5</v>
       </c>
       <c r="M9" t="n">
-        <v>94</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="10">
@@ -2959,25 +2959,25 @@
         <v>12</v>
       </c>
       <c r="G10" t="n">
-        <v>142</v>
+        <v>697</v>
       </c>
       <c r="H10" t="n">
-        <v>142</v>
+        <v>697</v>
       </c>
       <c r="I10" t="n">
-        <v>129</v>
+        <v>576</v>
       </c>
       <c r="J10" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="K10" t="n">
-        <v>14.8</v>
+        <v>31.5</v>
       </c>
       <c r="L10" t="n">
-        <v>182.2</v>
+        <v>219.7</v>
       </c>
       <c r="M10" t="n">
-        <v>80.59999999999999</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="11">
@@ -3007,28 +3007,28 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G11" t="n">
-        <v>2434</v>
+        <v>1465</v>
       </c>
       <c r="H11" t="n">
-        <v>2434</v>
+        <v>1465</v>
       </c>
       <c r="I11" t="n">
-        <v>2325</v>
+        <v>1300</v>
       </c>
       <c r="J11" t="n">
-        <v>109</v>
+        <v>162</v>
       </c>
       <c r="K11" t="n">
-        <v>5.7</v>
+        <v>17</v>
       </c>
       <c r="L11" t="n">
-        <v>114.6</v>
+        <v>152.4</v>
       </c>
       <c r="M11" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12">
@@ -3058,28 +3058,28 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="G12" t="n">
-        <v>241</v>
+        <v>2097</v>
       </c>
       <c r="H12" t="n">
-        <v>241</v>
+        <v>2097</v>
       </c>
       <c r="I12" t="n">
-        <v>232</v>
+        <v>1768</v>
       </c>
       <c r="J12" t="n">
-        <v>9</v>
+        <v>329</v>
       </c>
       <c r="K12" t="n">
-        <v>5.9</v>
+        <v>23.2</v>
       </c>
       <c r="L12" t="n">
-        <v>99</v>
+        <v>168.4</v>
       </c>
       <c r="M12" t="n">
-        <v>90.09999999999999</v>
+        <v>63.3</v>
       </c>
     </row>
     <row r="13">
@@ -3109,28 +3109,28 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G13" t="n">
-        <v>156</v>
+        <v>829</v>
       </c>
       <c r="H13" t="n">
-        <v>156</v>
+        <v>829</v>
       </c>
       <c r="I13" t="n">
-        <v>150</v>
+        <v>713</v>
       </c>
       <c r="J13" t="n">
-        <v>6</v>
+        <v>116</v>
       </c>
       <c r="K13" t="n">
-        <v>2.3</v>
+        <v>20.6</v>
       </c>
       <c r="L13" t="n">
-        <v>87.7</v>
+        <v>300.8</v>
       </c>
       <c r="M13" t="n">
-        <v>96</v>
+        <v>72.7</v>
       </c>
     </row>
     <row r="14">
@@ -3160,28 +3160,28 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="G14" t="n">
-        <v>2660</v>
+        <v>1570</v>
       </c>
       <c r="H14" t="n">
-        <v>2660</v>
+        <v>1570</v>
       </c>
       <c r="I14" t="n">
-        <v>2495</v>
+        <v>1415</v>
       </c>
       <c r="J14" t="n">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="K14" t="n">
-        <v>9.9</v>
+        <v>15.2</v>
       </c>
       <c r="L14" t="n">
-        <v>113.2</v>
+        <v>186.4</v>
       </c>
       <c r="M14" t="n">
-        <v>81.5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15">
@@ -3211,28 +3211,28 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="G15" t="n">
-        <v>257</v>
+        <v>2260</v>
       </c>
       <c r="H15" t="n">
-        <v>257</v>
+        <v>2260</v>
       </c>
       <c r="I15" t="n">
-        <v>243</v>
+        <v>1974</v>
       </c>
       <c r="J15" t="n">
-        <v>14</v>
+        <v>286</v>
       </c>
       <c r="K15" t="n">
-        <v>6.1</v>
+        <v>20.2</v>
       </c>
       <c r="L15" t="n">
-        <v>134.4</v>
+        <v>171</v>
       </c>
       <c r="M15" t="n">
-        <v>90.90000000000001</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16">
@@ -3265,25 +3265,25 @@
         <v>13</v>
       </c>
       <c r="G16" t="n">
-        <v>150</v>
+        <v>788</v>
       </c>
       <c r="H16" t="n">
-        <v>150</v>
+        <v>788</v>
       </c>
       <c r="I16" t="n">
-        <v>140</v>
+        <v>625</v>
       </c>
       <c r="J16" t="n">
-        <v>10</v>
+        <v>160</v>
       </c>
       <c r="K16" t="n">
-        <v>8.699999999999999</v>
+        <v>33</v>
       </c>
       <c r="L16" t="n">
-        <v>216.1</v>
+        <v>389.2</v>
       </c>
       <c r="M16" t="n">
-        <v>89.3</v>
+        <v>63.8</v>
       </c>
     </row>
     <row r="17">
@@ -3313,28 +3313,28 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="G17" t="n">
-        <v>2476</v>
+        <v>1631</v>
       </c>
       <c r="H17" t="n">
-        <v>2476</v>
+        <v>1631</v>
       </c>
       <c r="I17" t="n">
-        <v>2400</v>
+        <v>1392</v>
       </c>
       <c r="J17" t="n">
-        <v>76</v>
+        <v>239</v>
       </c>
       <c r="K17" t="n">
-        <v>4.5</v>
+        <v>23.7</v>
       </c>
       <c r="L17" t="n">
-        <v>119.8</v>
+        <v>210.6</v>
       </c>
       <c r="M17" t="n">
-        <v>92.2</v>
+        <v>65.5</v>
       </c>
     </row>
     <row r="18">
@@ -3364,28 +3364,28 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="G18" t="n">
-        <v>232</v>
+        <v>2214</v>
       </c>
       <c r="H18" t="n">
-        <v>232</v>
+        <v>2214</v>
       </c>
       <c r="I18" t="n">
-        <v>229</v>
+        <v>1939</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>275</v>
       </c>
       <c r="K18" t="n">
-        <v>5.1</v>
+        <v>20.9</v>
       </c>
       <c r="L18" t="n">
-        <v>146.5</v>
+        <v>187</v>
       </c>
       <c r="M18" t="n">
-        <v>93</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="19">
@@ -3415,28 +3415,28 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G19" t="n">
-        <v>153</v>
+        <v>861</v>
       </c>
       <c r="H19" t="n">
-        <v>153</v>
+        <v>861</v>
       </c>
       <c r="I19" t="n">
-        <v>144</v>
+        <v>656</v>
       </c>
       <c r="J19" t="n">
-        <v>9</v>
+        <v>205</v>
       </c>
       <c r="K19" t="n">
-        <v>9.699999999999999</v>
+        <v>35.6</v>
       </c>
       <c r="L19" t="n">
-        <v>138.6</v>
+        <v>269.5</v>
       </c>
       <c r="M19" t="n">
-        <v>88.2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20">
@@ -3466,28 +3466,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="G20" t="n">
-        <v>2599</v>
+        <v>1869</v>
       </c>
       <c r="H20" t="n">
-        <v>2599</v>
+        <v>1869</v>
       </c>
       <c r="I20" t="n">
-        <v>2479</v>
+        <v>1597</v>
       </c>
       <c r="J20" t="n">
-        <v>120</v>
+        <v>272</v>
       </c>
       <c r="K20" t="n">
-        <v>7.2</v>
+        <v>22.8</v>
       </c>
       <c r="L20" t="n">
-        <v>145.9</v>
+        <v>184.7</v>
       </c>
       <c r="M20" t="n">
-        <v>86.2</v>
+        <v>62.9</v>
       </c>
     </row>
     <row r="21">
@@ -3517,28 +3517,28 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G21" t="n">
-        <v>248</v>
+        <v>2173</v>
       </c>
       <c r="H21" t="n">
-        <v>248</v>
+        <v>2173</v>
       </c>
       <c r="I21" t="n">
-        <v>240</v>
+        <v>1897</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>276</v>
       </c>
       <c r="K21" t="n">
-        <v>7.8</v>
+        <v>20</v>
       </c>
       <c r="L21" t="n">
-        <v>101.4</v>
+        <v>161</v>
       </c>
       <c r="M21" t="n">
-        <v>85.40000000000001</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="22">
@@ -3568,28 +3568,28 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G22" t="n">
-        <v>162</v>
+        <v>887</v>
       </c>
       <c r="H22" t="n">
-        <v>162</v>
+        <v>887</v>
       </c>
       <c r="I22" t="n">
-        <v>150</v>
+        <v>810</v>
       </c>
       <c r="J22" t="n">
-        <v>9</v>
+        <v>77</v>
       </c>
       <c r="K22" t="n">
-        <v>5.1</v>
+        <v>12.3</v>
       </c>
       <c r="L22" t="n">
-        <v>137.1</v>
+        <v>168.6</v>
       </c>
       <c r="M22" t="n">
-        <v>92</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -3619,28 +3619,28 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="G23" t="n">
-        <v>2974</v>
+        <v>1528</v>
       </c>
       <c r="H23" t="n">
-        <v>2974</v>
+        <v>1528</v>
       </c>
       <c r="I23" t="n">
-        <v>2821</v>
+        <v>1354</v>
       </c>
       <c r="J23" t="n">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="K23" t="n">
-        <v>8.199999999999999</v>
+        <v>16.4</v>
       </c>
       <c r="L23" t="n">
-        <v>129.5</v>
+        <v>191.4</v>
       </c>
       <c r="M23" t="n">
-        <v>84.09999999999999</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24">
@@ -3670,28 +3670,28 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G24" t="n">
-        <v>276</v>
+        <v>1880</v>
       </c>
       <c r="H24" t="n">
-        <v>276</v>
+        <v>1880</v>
       </c>
       <c r="I24" t="n">
-        <v>261</v>
+        <v>1607</v>
       </c>
       <c r="J24" t="n">
-        <v>15</v>
+        <v>273</v>
       </c>
       <c r="K24" t="n">
-        <v>4.7</v>
+        <v>24.3</v>
       </c>
       <c r="L24" t="n">
-        <v>107.4</v>
+        <v>198.1</v>
       </c>
       <c r="M24" t="n">
-        <v>92.3</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="27">
@@ -3753,25 +3753,25 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1530</v>
+        <v>2399</v>
       </c>
       <c r="C30" t="n">
-        <v>1530</v>
+        <v>2399</v>
       </c>
       <c r="D30" t="n">
-        <v>1437</v>
+        <v>1974</v>
       </c>
       <c r="E30" t="n">
-        <v>93</v>
+        <v>425</v>
       </c>
       <c r="F30" t="n">
-        <v>6.1</v>
+        <v>17.7</v>
       </c>
       <c r="G30" t="n">
-        <v>89.7</v>
+        <v>66.8</v>
       </c>
       <c r="H30" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31">
@@ -3781,25 +3781,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3177</v>
+        <v>2604</v>
       </c>
       <c r="C31" t="n">
-        <v>3177</v>
+        <v>2604</v>
       </c>
       <c r="D31" t="n">
-        <v>3038</v>
+        <v>2181</v>
       </c>
       <c r="E31" t="n">
-        <v>139</v>
+        <v>423</v>
       </c>
       <c r="F31" t="n">
-        <v>4.4</v>
+        <v>16.2</v>
       </c>
       <c r="G31" t="n">
-        <v>91.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32">
@@ -3809,25 +3809,25 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2817</v>
+        <v>4259</v>
       </c>
       <c r="C32" t="n">
-        <v>2817</v>
+        <v>4259</v>
       </c>
       <c r="D32" t="n">
-        <v>2686</v>
+        <v>3644</v>
       </c>
       <c r="E32" t="n">
-        <v>131</v>
+        <v>610</v>
       </c>
       <c r="F32" t="n">
-        <v>4.7</v>
+        <v>14.3</v>
       </c>
       <c r="G32" t="n">
-        <v>86.90000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="H32" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33">
@@ -3837,25 +3837,25 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3073</v>
+        <v>4659</v>
       </c>
       <c r="C33" t="n">
-        <v>3073</v>
+        <v>4659</v>
       </c>
       <c r="D33" t="n">
-        <v>2888</v>
+        <v>4102</v>
       </c>
       <c r="E33" t="n">
-        <v>185</v>
+        <v>557</v>
       </c>
       <c r="F33" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G33" t="n">
-        <v>89.5</v>
+        <v>72.2</v>
       </c>
       <c r="H33" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34">
@@ -3865,25 +3865,25 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2858</v>
+        <v>4633</v>
       </c>
       <c r="C34" t="n">
-        <v>2858</v>
+        <v>4633</v>
       </c>
       <c r="D34" t="n">
-        <v>2769</v>
+        <v>3956</v>
       </c>
       <c r="E34" t="n">
-        <v>89</v>
+        <v>674</v>
       </c>
       <c r="F34" t="n">
-        <v>3.1</v>
+        <v>14.5</v>
       </c>
       <c r="G34" t="n">
-        <v>91.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="H34" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35">
@@ -3893,25 +3893,25 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3000</v>
+        <v>4903</v>
       </c>
       <c r="C35" t="n">
-        <v>3000</v>
+        <v>4903</v>
       </c>
       <c r="D35" t="n">
-        <v>2863</v>
+        <v>4150</v>
       </c>
       <c r="E35" t="n">
-        <v>137</v>
+        <v>753</v>
       </c>
       <c r="F35" t="n">
-        <v>4.6</v>
+        <v>15.4</v>
       </c>
       <c r="G35" t="n">
-        <v>86.59999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36">
@@ -3921,25 +3921,25 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3412</v>
+        <v>4295</v>
       </c>
       <c r="C36" t="n">
-        <v>3412</v>
+        <v>4295</v>
       </c>
       <c r="D36" t="n">
-        <v>3232</v>
+        <v>3771</v>
       </c>
       <c r="E36" t="n">
-        <v>177</v>
+        <v>524</v>
       </c>
       <c r="F36" t="n">
-        <v>5.2</v>
+        <v>12.2</v>
       </c>
       <c r="G36" t="n">
-        <v>89.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37">
@@ -3949,25 +3949,25 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>19867</v>
+        <v>27752</v>
       </c>
       <c r="C37" t="n">
-        <v>19867</v>
+        <v>27752</v>
       </c>
       <c r="D37" t="n">
-        <v>18913</v>
+        <v>23778</v>
       </c>
       <c r="E37" t="n">
-        <v>951</v>
+        <v>3966</v>
       </c>
       <c r="F37" t="n">
-        <v>4.8</v>
+        <v>14.3</v>
       </c>
       <c r="G37" t="n">
-        <v>89.3</v>
+        <v>68.2</v>
       </c>
       <c r="H37" t="n">
-        <v>566</v>
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -4088,28 +4088,28 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G4" t="n">
-        <v>129</v>
+        <v>782</v>
       </c>
       <c r="H4" t="n">
-        <v>129</v>
+        <v>782</v>
       </c>
       <c r="I4" t="n">
-        <v>123</v>
+        <v>777</v>
       </c>
       <c r="J4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K4" t="n">
-        <v>4.1</v>
+        <v>0.9</v>
       </c>
       <c r="L4" t="n">
-        <v>228.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>97.59999999999999</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -4139,28 +4139,28 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G5" t="n">
-        <v>1319</v>
+        <v>795</v>
       </c>
       <c r="H5" t="n">
-        <v>1319</v>
+        <v>795</v>
       </c>
       <c r="I5" t="n">
-        <v>1293</v>
+        <v>789</v>
       </c>
       <c r="J5" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="K5" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="L5" t="n">
-        <v>113.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>95.5</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="6">
@@ -4190,28 +4190,28 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="H6" t="n">
-        <v>82</v>
+        <v>822</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>792</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="K6" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="L6" t="n">
-        <v>98</v>
+        <v>206.3</v>
       </c>
       <c r="M6" t="n">
-        <v>96.2</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -4241,28 +4241,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>119</v>
+        <v>167</v>
       </c>
       <c r="H7" t="n">
-        <v>119</v>
+        <v>167</v>
       </c>
       <c r="I7" t="n">
-        <v>113</v>
+        <v>164</v>
       </c>
       <c r="J7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L7" t="n">
-        <v>89.40000000000001</v>
+        <v>204.1</v>
       </c>
       <c r="M7" t="n">
-        <v>97.3</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="8">
@@ -4292,28 +4292,28 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="G8" t="n">
-        <v>2781</v>
+        <v>913</v>
       </c>
       <c r="H8" t="n">
-        <v>2781</v>
+        <v>913</v>
       </c>
       <c r="I8" t="n">
-        <v>2749</v>
+        <v>896</v>
       </c>
       <c r="J8" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="K8" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="L8" t="n">
-        <v>67.5</v>
+        <v>56.1</v>
       </c>
       <c r="M8" t="n">
-        <v>95.2</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9">
@@ -4343,28 +4343,28 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="G9" t="n">
-        <v>277</v>
+        <v>1524</v>
       </c>
       <c r="H9" t="n">
-        <v>277</v>
+        <v>1524</v>
       </c>
       <c r="I9" t="n">
-        <v>271</v>
+        <v>1504</v>
       </c>
       <c r="J9" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K9" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="L9" t="n">
-        <v>68.3</v>
+        <v>67.5</v>
       </c>
       <c r="M9" t="n">
-        <v>95.59999999999999</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
@@ -4394,28 +4394,28 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G10" t="n">
-        <v>142</v>
+        <v>697</v>
       </c>
       <c r="H10" t="n">
-        <v>142</v>
+        <v>697</v>
       </c>
       <c r="I10" t="n">
-        <v>137</v>
+        <v>691</v>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" t="n">
-        <v>4.5</v>
+        <v>0.9</v>
       </c>
       <c r="L10" t="n">
-        <v>229.9</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>95.59999999999999</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="11">
@@ -4445,28 +4445,28 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="G11" t="n">
-        <v>2434</v>
+        <v>1465</v>
       </c>
       <c r="H11" t="n">
-        <v>2434</v>
+        <v>1465</v>
       </c>
       <c r="I11" t="n">
-        <v>2379</v>
+        <v>1446</v>
       </c>
       <c r="J11" t="n">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="K11" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="L11" t="n">
-        <v>88.7</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>95.2</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -4496,28 +4496,28 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>241</v>
+        <v>2097</v>
       </c>
       <c r="H12" t="n">
-        <v>241</v>
+        <v>2097</v>
       </c>
       <c r="I12" t="n">
-        <v>239</v>
+        <v>2060</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="K12" t="n">
-        <v>1.1</v>
+        <v>2.7</v>
       </c>
       <c r="L12" t="n">
-        <v>41.3</v>
+        <v>101.7</v>
       </c>
       <c r="M12" t="n">
-        <v>97.5</v>
+        <v>95.09999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -4547,28 +4547,28 @@
         </is>
       </c>
       <c r="F13" t="n">
+        <v>21</v>
+      </c>
+      <c r="G13" t="n">
+        <v>829</v>
+      </c>
+      <c r="H13" t="n">
+        <v>829</v>
+      </c>
+      <c r="I13" t="n">
+        <v>816</v>
+      </c>
+      <c r="J13" t="n">
         <v>13</v>
       </c>
-      <c r="G13" t="n">
-        <v>156</v>
-      </c>
-      <c r="H13" t="n">
-        <v>156</v>
-      </c>
-      <c r="I13" t="n">
-        <v>150</v>
-      </c>
-      <c r="J13" t="n">
-        <v>6</v>
-      </c>
       <c r="K13" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="L13" t="n">
-        <v>87.7</v>
+        <v>75.8</v>
       </c>
       <c r="M13" t="n">
-        <v>96</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -4598,28 +4598,28 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="G14" t="n">
-        <v>2660</v>
+        <v>1570</v>
       </c>
       <c r="H14" t="n">
-        <v>2660</v>
+        <v>1570</v>
       </c>
       <c r="I14" t="n">
-        <v>2622</v>
+        <v>1536</v>
       </c>
       <c r="J14" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="K14" t="n">
-        <v>1.9</v>
+        <v>2.9</v>
       </c>
       <c r="L14" t="n">
-        <v>56.5</v>
+        <v>93.7</v>
       </c>
       <c r="M14" t="n">
-        <v>96.2</v>
+        <v>95.09999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -4649,28 +4649,28 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="G15" t="n">
-        <v>257</v>
+        <v>2260</v>
       </c>
       <c r="H15" t="n">
-        <v>257</v>
+        <v>2260</v>
       </c>
       <c r="I15" t="n">
-        <v>252</v>
+        <v>2217</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="K15" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="L15" t="n">
-        <v>91.7</v>
+        <v>135.2</v>
       </c>
       <c r="M15" t="n">
-        <v>96.40000000000001</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="16">
@@ -4700,28 +4700,28 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G16" t="n">
-        <v>150</v>
+        <v>788</v>
       </c>
       <c r="H16" t="n">
-        <v>150</v>
+        <v>788</v>
       </c>
       <c r="I16" t="n">
-        <v>145</v>
+        <v>776</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K16" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="L16" t="n">
-        <v>73.09999999999999</v>
+        <v>100.6</v>
       </c>
       <c r="M16" t="n">
-        <v>97.2</v>
+        <v>95.59999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -4751,28 +4751,28 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="G17" t="n">
-        <v>2476</v>
+        <v>1631</v>
       </c>
       <c r="H17" t="n">
-        <v>2476</v>
+        <v>1631</v>
       </c>
       <c r="I17" t="n">
-        <v>2437</v>
+        <v>1616</v>
       </c>
       <c r="J17" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="K17" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="L17" t="n">
-        <v>113.2</v>
+        <v>68.5</v>
       </c>
       <c r="M17" t="n">
-        <v>95.2</v>
+        <v>96.40000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -4802,28 +4802,28 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="G18" t="n">
-        <v>232</v>
+        <v>2214</v>
       </c>
       <c r="H18" t="n">
-        <v>232</v>
+        <v>2214</v>
       </c>
       <c r="I18" t="n">
-        <v>229</v>
+        <v>2186</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="K18" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="L18" t="n">
-        <v>122</v>
+        <v>79</v>
       </c>
       <c r="M18" t="n">
-        <v>97.40000000000001</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -4853,28 +4853,28 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G19" t="n">
-        <v>153</v>
+        <v>861</v>
       </c>
       <c r="H19" t="n">
-        <v>153</v>
+        <v>861</v>
       </c>
       <c r="I19" t="n">
-        <v>147</v>
+        <v>848</v>
       </c>
       <c r="J19" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="K19" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="L19" t="n">
-        <v>120.8</v>
+        <v>135.5</v>
       </c>
       <c r="M19" t="n">
-        <v>98</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="20">
@@ -4904,28 +4904,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G20" t="n">
-        <v>2599</v>
+        <v>1869</v>
       </c>
       <c r="H20" t="n">
-        <v>2599</v>
+        <v>1869</v>
       </c>
       <c r="I20" t="n">
-        <v>2556</v>
+        <v>1842</v>
       </c>
       <c r="J20" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="K20" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="L20" t="n">
-        <v>94.90000000000001</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>95.2</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="21">
@@ -4955,28 +4955,28 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="G21" t="n">
-        <v>248</v>
+        <v>2173</v>
       </c>
       <c r="H21" t="n">
-        <v>248</v>
+        <v>2173</v>
       </c>
       <c r="I21" t="n">
-        <v>247</v>
+        <v>2142</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="K21" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="L21" t="n">
-        <v>46.4</v>
+        <v>97.2</v>
       </c>
       <c r="M21" t="n">
-        <v>97.2</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -5006,28 +5006,28 @@
         </is>
       </c>
       <c r="F22" t="n">
+        <v>23</v>
+      </c>
+      <c r="G22" t="n">
+        <v>887</v>
+      </c>
+      <c r="H22" t="n">
+        <v>887</v>
+      </c>
+      <c r="I22" t="n">
+        <v>872</v>
+      </c>
+      <c r="J22" t="n">
         <v>15</v>
       </c>
-      <c r="G22" t="n">
-        <v>162</v>
-      </c>
-      <c r="H22" t="n">
-        <v>162</v>
-      </c>
-      <c r="I22" t="n">
-        <v>162</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
       <c r="K22" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="L22" t="n">
-        <v>17.1</v>
+        <v>95.8</v>
       </c>
       <c r="M22" t="n">
-        <v>100</v>
+        <v>97.90000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -5057,28 +5057,28 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="G23" t="n">
-        <v>2974</v>
+        <v>1528</v>
       </c>
       <c r="H23" t="n">
-        <v>2974</v>
+        <v>1528</v>
       </c>
       <c r="I23" t="n">
-        <v>2946</v>
+        <v>1495</v>
       </c>
       <c r="J23" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="K23" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="L23" t="n">
-        <v>71.59999999999999</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>96.09999999999999</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="24">
@@ -5108,28 +5108,28 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="G24" t="n">
-        <v>276</v>
+        <v>1880</v>
       </c>
       <c r="H24" t="n">
-        <v>276</v>
+        <v>1880</v>
       </c>
       <c r="I24" t="n">
-        <v>265</v>
+        <v>1855</v>
       </c>
       <c r="J24" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="K24" t="n">
-        <v>3.1</v>
+        <v>2.1</v>
       </c>
       <c r="L24" t="n">
-        <v>105.2</v>
+        <v>72</v>
       </c>
       <c r="M24" t="n">
-        <v>95.09999999999999</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="27">
@@ -5191,25 +5191,25 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1530</v>
+        <v>2399</v>
       </c>
       <c r="C30" t="n">
-        <v>1530</v>
+        <v>2399</v>
       </c>
       <c r="D30" t="n">
-        <v>1496</v>
+        <v>2358</v>
       </c>
       <c r="E30" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F30" t="n">
-        <v>2.2</v>
+        <v>1.7</v>
       </c>
       <c r="G30" t="n">
-        <v>96.40000000000001</v>
+        <v>97</v>
       </c>
       <c r="H30" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31">
@@ -5219,25 +5219,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3177</v>
+        <v>2604</v>
       </c>
       <c r="C31" t="n">
-        <v>3177</v>
+        <v>2604</v>
       </c>
       <c r="D31" t="n">
-        <v>3133</v>
+        <v>2564</v>
       </c>
       <c r="E31" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F31" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="G31" t="n">
-        <v>96</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32">
@@ -5247,25 +5247,25 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2817</v>
+        <v>4259</v>
       </c>
       <c r="C32" t="n">
-        <v>2817</v>
+        <v>4259</v>
       </c>
       <c r="D32" t="n">
-        <v>2755</v>
+        <v>4197</v>
       </c>
       <c r="E32" t="n">
         <v>62</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="G32" t="n">
-        <v>96.09999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="H32" t="n">
-        <v>91</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33">
@@ -5275,25 +5275,25 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3073</v>
+        <v>4659</v>
       </c>
       <c r="C33" t="n">
-        <v>3073</v>
+        <v>4659</v>
       </c>
       <c r="D33" t="n">
-        <v>3024</v>
+        <v>4569</v>
       </c>
       <c r="E33" t="n">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="F33" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="G33" t="n">
-        <v>96.2</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H33" t="n">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34">
@@ -5303,25 +5303,25 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2858</v>
+        <v>4633</v>
       </c>
       <c r="C34" t="n">
-        <v>2858</v>
+        <v>4633</v>
       </c>
       <c r="D34" t="n">
-        <v>2811</v>
+        <v>4578</v>
       </c>
       <c r="E34" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F34" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="G34" t="n">
-        <v>96.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="H34" t="n">
-        <v>91</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35">
@@ -5331,25 +5331,25 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3000</v>
+        <v>4903</v>
       </c>
       <c r="C35" t="n">
-        <v>3000</v>
+        <v>4903</v>
       </c>
       <c r="D35" t="n">
-        <v>2950</v>
+        <v>4832</v>
       </c>
       <c r="E35" t="n">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="F35" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="G35" t="n">
-        <v>96.8</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>97</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36">
@@ -5359,25 +5359,25 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3412</v>
+        <v>4295</v>
       </c>
       <c r="C36" t="n">
-        <v>3412</v>
+        <v>4295</v>
       </c>
       <c r="D36" t="n">
-        <v>3373</v>
+        <v>4222</v>
       </c>
       <c r="E36" t="n">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="F36" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G36" t="n">
-        <v>97.09999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37">
@@ -5387,16 +5387,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>19867</v>
+        <v>27752</v>
       </c>
       <c r="C37" t="n">
-        <v>19867</v>
+        <v>27752</v>
       </c>
       <c r="D37" t="n">
-        <v>19542</v>
+        <v>27320</v>
       </c>
       <c r="E37" t="n">
-        <v>325</v>
+        <v>432</v>
       </c>
       <c r="F37" t="n">
         <v>1.6</v>
@@ -5405,7 +5405,7 @@
         <v>96.5</v>
       </c>
       <c r="H37" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
     </row>
     <row r="40">
@@ -5462,22 +5462,22 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C43" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D43" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E43" t="n">
-        <v>89.7</v>
+        <v>66.8</v>
       </c>
       <c r="F43" t="n">
-        <v>96.40000000000001</v>
+        <v>97</v>
       </c>
       <c r="G43" t="n">
-        <v>6.7</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="44">
@@ -5487,22 +5487,22 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="C44" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E44" t="n">
-        <v>91.40000000000001</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="F44" t="n">
-        <v>96</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="G44" t="n">
-        <v>4.6</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="45">
@@ -5512,22 +5512,22 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C45" t="n">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="E45" t="n">
-        <v>86.90000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F45" t="n">
-        <v>96.09999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="G45" t="n">
-        <v>9.199999999999999</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="46">
@@ -5537,22 +5537,22 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C46" t="n">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="D46" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E46" t="n">
-        <v>89.5</v>
+        <v>72.2</v>
       </c>
       <c r="F46" t="n">
-        <v>96.2</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="G46" t="n">
-        <v>6.7</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="47">
@@ -5562,22 +5562,22 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C47" t="n">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="D47" t="n">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="E47" t="n">
-        <v>91.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F47" t="n">
-        <v>96.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="G47" t="n">
-        <v>5.1</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="48">
@@ -5587,22 +5587,22 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C48" t="n">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="D48" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="E48" t="n">
-        <v>86.59999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F48" t="n">
-        <v>96.8</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>10.2</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="49">
@@ -5612,22 +5612,22 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C49" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D49" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E49" t="n">
-        <v>89.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F49" t="n">
-        <v>97.09999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G49" t="n">
-        <v>7.6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50">
@@ -5637,22 +5637,22 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>566</v>
+        <v>526</v>
       </c>
       <c r="C50" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
       <c r="D50" t="n">
-        <v>70</v>
+        <v>219</v>
       </c>
       <c r="E50" t="n">
-        <v>89.3</v>
+        <v>68.2</v>
       </c>
       <c r="F50" t="n">
         <v>96.5</v>
       </c>
       <c r="G50" t="n">
-        <v>7.2</v>
+        <v>28.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>